<commit_message>
결과 파일 업데이트 2026-08-21 08:33
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260821.xlsx
+++ b/results/andar_할인율모니터링_20260821.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H171"/>
+  <dimension ref="A1:H172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,7 +491,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>7,435</t>
+          <t>7,445</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4,998</t>
+          <t>5,001</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -575,7 +575,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>307</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>307</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>307</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -671,42 +671,42 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17407&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10940&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EPTBG-04</t>
+          <t>ENTBG-03</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>드라이 페더 버킷백</t>
+          <t>데일리 스트링 쇼퍼백</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>55,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>680</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1,881</t>
+          <t>1,882</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>1,881</t>
+          <t>1,882</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>1,881</t>
+          <t>1,882</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>72</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>138</t>
+          <t>139</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1343,42 +1343,42 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10940&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17407&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ENTBG-03</t>
+          <t>EPTBG-04</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>데일리 스트링 쇼퍼백</t>
+          <t>드라이 페더 버킷백</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>55,000</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>680</t>
+          <t>75</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2,225</t>
+          <t>2,226</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1511,42 +1511,42 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15432&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16868&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ENTSC-12</t>
+          <t>EPTBG-03</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 퍼포먼스 토삭스</t>
+          <t>컴팩트 포켓 크로스백</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>25,800</t>
+          <t>65,000</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>3,437</t>
+          <t>94</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EOTSC-15</t>
+          <t>ENTSC-12</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>3,437</t>
+          <t>3,439</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1595,42 +1595,42 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16868&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15432&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>EPTBG-03</t>
+          <t>EOTSC-15</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>컴팩트 포켓 크로스백</t>
+          <t>[1&amp;1] 논슬립 퍼포먼스 토삭스</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>65,000</t>
+          <t>25,800</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>3,439</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>69</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1721,37 +1721,37 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15372&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12488&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>EOTBG-16</t>
+          <t>ENTBG-10</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>폴더블 미니백 2.0</t>
+          <t>스퀘어 크로스백</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>596</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -1763,37 +1763,37 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12488&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15372&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ENTBG-10</t>
+          <t>EOTBG-16</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>스퀘어 크로스백</t>
+          <t>폴더블 미니백 2.0</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>595</t>
+          <t>238</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1931,84 +1931,84 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6952&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15403&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>EJFST-02</t>
+          <t>EOTBG-21</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>릴렉스 요가링</t>
+          <t>데일리 라운드백</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>75,000</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>3,900</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>6,502</t>
+          <t>83</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15403&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6952&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>EOTBG-21</t>
+          <t>EJFST-02</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>데일리 라운드백</t>
+          <t>릴렉스 요가링</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>75,000</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>3,900</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>6,502</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>405</t>
+          <t>406</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>4,779</t>
+          <t>4,781</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2561,79 +2561,79 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9989&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EMTET-02</t>
+          <t>EOTSV-04</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>소프트 쿠셔닝 훌라후프</t>
+          <t>[3 PCS] 러닝 용품 올인원 세트 (러닝 밴드 &amp; 무릎 보호대 &amp; 삭스)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>57,800</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>15,000</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>591</t>
+          <t>1,545</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>EMTSC-04</t>
+          <t>EOTSV-01</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
+          <t>[3 PCS] 러닝 용품 올인원 세트 (러닝 밴드 &amp; 무릎 보호대 &amp; 삭스)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>19,800</t>
+          <t>57,800</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>3,149</t>
+          <t>1,545</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -2645,37 +2645,37 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EMTSC-05</t>
+          <t>EOTSC-06</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
+          <t>[3 PCS] 러닝 용품 올인원 세트 (러닝 밴드 &amp; 무릎 보호대 &amp; 삭스)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>19,800</t>
+          <t>57,800</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>3,149</t>
+          <t>1,545</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -2687,37 +2687,37 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13853&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9989&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EOTBG-12</t>
+          <t>EMTET-02</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>프리런 벨크로 러닝 벨트</t>
+          <t>소프트 쿠셔닝 훌라후프</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>15,000</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>592</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -2729,79 +2729,79 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11110&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ENTCP-01</t>
+          <t>EMTSC-04</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>와이드 셰이드 버킷햇</t>
+          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>51%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>681</t>
+          <t>3,149</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8819&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EOTSV-04</t>
+          <t>EMTSC-05</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>[3 PCS] 러닝 용품 올인원 세트 (러닝 밴드 &amp; 무릎 보호대 &amp; 삭스)</t>
+          <t>[1&amp;1] 논슬립 서포트 하프 토삭스 (HOLE &amp; SOLID)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>57,800</t>
+          <t>19,800</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>1,545</t>
+          <t>3,149</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -2813,7 +2813,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13604&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2823,17 +2823,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>[3 PCS] 러닝 용품 올인원 세트 (러닝 밴드 &amp; 무릎 보호대 &amp; 삭스)</t>
+          <t>[1&amp;1] 하이 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>57,800</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2843,91 +2843,91 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>1,545</t>
+          <t>672</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13853&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EOTSC-06</t>
+          <t>EOTBG-12</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>[3 PCS] 러닝 용품 올인원 세트 (러닝 밴드 &amp; 무릎 보호대 &amp; 삭스)</t>
+          <t>프리런 벨크로 러닝 벨트</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>57,800</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>17%</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>1,545</t>
+          <t>230</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13604&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11110&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EOTSV-01</t>
+          <t>ENTCP-01</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>[1&amp;1] 하이 서포트 무릎 보호대</t>
+          <t>와이드 셰이드 버킷햇</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>51%</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>672</t>
+          <t>681</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -2981,84 +2981,84 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15629&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14085&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EOTBG-23</t>
+          <t>EOTSV-04</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>안다르 실버 리유저블백 M</t>
+          <t>프리런 라이트 러닝 밴드</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>22,000</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>337</t>
+          <t>122</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.2</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14085&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15629&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EOTSV-04</t>
+          <t>EOTBG-23</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>프리런 라이트 러닝 밴드</t>
+          <t>안다르 실버 리유저블백 M</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>22,000</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>337</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>209</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3107,79 +3107,79 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16844&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15143&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EPTET-02</t>
+          <t>EOTBG-17</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>언더웨어 세탁망</t>
+          <t>3 in 1 캐리온 더플백</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>109,000</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>89,000</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>266</t>
+          <t>37</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15143&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15350&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EOTBG-17</t>
+          <t>EOTSC-09</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>3 in 1 캐리온 더플백</t>
+          <t>[1&amp;1] 컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>109,000</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>89,000</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>642</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3191,42 +3191,42 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15350&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16844&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>EOTSC-09</t>
+          <t>EPTET-02</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>[1&amp;1] 컴프레션 러닝 니삭스</t>
+          <t>언더웨어 세탁망</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>642</t>
+          <t>266</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>1,526</t>
+          <t>1,528</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3317,84 +3317,84 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8621&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EMTSV-06</t>
+          <t>EPTFB-02</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>에어쿨링 손목 보호대</t>
+          <t>퍼포먼스 심리스 손목밴드</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>1,069</t>
+          <t>213</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8621&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EPTFB-02</t>
+          <t>EMTSV-06</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>퍼포먼스 심리스 손목밴드</t>
+          <t>에어쿨링 손목 보호대</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>211</t>
+          <t>1,069</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3515,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>4,779</t>
+          <t>4,781</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3611,37 +3611,37 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16632&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16847&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EPTSV-02</t>
+          <t>EPTSC-02</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>[1&amp;1] 하이 서포트 발목 보호대</t>
+          <t>하이 쿠션 테이핑 러닝 삭스</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>79</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -3653,42 +3653,42 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16632&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>EMTRB-01</t>
+          <t>EPTSV-02</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>서포트 힙 밴드</t>
+          <t>[1&amp;1] 하이 서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>1,349</t>
+          <t>99</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -3700,7 +3700,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>EMTRB-02</t>
+          <t>EMTRB-01</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3742,7 +3742,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>EMTRB-03</t>
+          <t>EMTRB-02</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3779,79 +3779,79 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16847&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>EPTSC-02</t>
+          <t>EMTRB-03</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>하이 쿠션 테이핑 러닝 삭스</t>
+          <t>서포트 힙 밴드</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>1,349</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11039&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>EOTGL-01</t>
+          <t>ENTFB-01</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>짐 글러브 2.0</t>
+          <t>에어쿨링 라인 스크런치</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>21,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>11%</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>718</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -3863,37 +3863,37 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11039&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ENTFB-01</t>
+          <t>EOTGL-01</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>에어쿨링 라인 스크런치</t>
+          <t>짐 글러브 2.0</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>21,000</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>11%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>716</t>
+          <t>270</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -4031,121 +4031,121 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11027&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15377&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ENTSC-08</t>
+          <t>EOTGL-04</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>[5 SET] 에어컴피 크루 삭스</t>
+          <t>논슬립 스킨 요기 글러브</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>85,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>35,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>59%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>804</t>
+          <t>172</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15377&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11027&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EOTGL-04</t>
+          <t>ENTSC-08</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>논슬립 스킨 요기 글러브</t>
+          <t>[5 SET] 에어컴피 크루 삭스</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>85,000</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>35,000</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>59%</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>804</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10554&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>ENTMK-01</t>
+          <t>EOTSC-16</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>UV 프로텍션 맨즈 골프 마스크</t>
+          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>25,800</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>15,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>1,523</t>
+          <t>486</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -4157,69 +4157,69 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EOTSC-09</t>
+          <t>EOTSC-17</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>컴프레션 러닝 니삭스</t>
+          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>25,800</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>333</t>
+          <t>486</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15408&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EOTSC-14</t>
+          <t>EOTSC-09</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>맨즈 논슬립 풀 토삭스</t>
+          <t>컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4229,91 +4229,91 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>333</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15408&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EOTSC-16</t>
+          <t>EOTSC-14</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
+          <t>맨즈 논슬립 풀 토삭스</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>25,800</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>485</t>
+          <t>96</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10554&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EOTSC-17</t>
+          <t>ENTMK-01</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
+          <t>UV 프로텍션 맨즈 골프 마스크</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>25,800</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>15,000</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>485</t>
+          <t>1,523</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4325,84 +4325,84 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=5837&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15153&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EJFMB-03</t>
+          <t>EOTSC-13</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>릴렉스 짐볼 65cm</t>
+          <t>테이핑 테크 러닝 삭스</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>2,082</t>
+          <t>260</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15153&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=5837&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EOTSC-13</t>
+          <t>EJFMB-03</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>테이핑 테크 러닝 삭스</t>
+          <t>릴렉스 짐볼 65cm</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>260</t>
+          <t>2,082</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -4451,69 +4451,69 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11456&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ENTSC-13</t>
+          <t>EKPMB-02</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 퍼포먼스 삭스</t>
+          <t>릴렉스 미니 짐볼</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>17,800</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>3,002</t>
+          <t>1,215</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11456&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8578&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ENTSC-14</t>
+          <t>EMTSC-01</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 퍼포먼스 삭스</t>
+          <t>링글 크루 삭스</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>17,800</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4523,81 +4523,81 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>3,002</t>
+          <t>1,313</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11456&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>EKPMB-02</t>
+          <t>ENTSC-13</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>릴렉스 미니 짐볼</t>
+          <t>[1&amp;1] 논슬립 퍼포먼스 삭스</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>17,800</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>1,215</t>
+          <t>3,003</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8578&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11456&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>EMTSC-01</t>
+          <t>ENTSC-14</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>링글 크루 삭스</t>
+          <t>[1&amp;1] 논슬립 퍼포먼스 삭스</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>17,800</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4607,12 +4607,12 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>1,313</t>
+          <t>3,003</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -4703,111 +4703,111 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14084&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17446&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EOTET-01</t>
+          <t>EPTSV-01</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>소프트 뱀부 롱 타월</t>
+          <t>[1&amp;1] 3D 쿨링 핑거홀 팔토시</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>31,800</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>24,900</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>227</t>
+          <t>176</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13405&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16640&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>EOTSV-01</t>
+          <t>EPTBG-05</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>하이 서포트 무릎 보호대</t>
+          <t>안다르 시그니처 로고 에코백</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>672</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16640&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14084&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>EPTBG-05</t>
+          <t>EOTET-01</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>안다르 시그니처 로고 에코백</t>
+          <t>소프트 뱀부 롱 타월</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4817,217 +4817,217 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>227</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17446&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6828&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>EPTSV-01</t>
+          <t>EKPET-01</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>[1&amp;1] 3D 쿨링 핑거홀 팔토시</t>
+          <t>[1&amp;1] 릴렉스 소프트 웨이트바 1kg</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>31,800</t>
+          <t>41,800</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>24,900</t>
+          <t>35,600</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>176</t>
+          <t>590</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6828&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8837&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>EKPET-01</t>
+          <t>EMTSV-02</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>[1&amp;1] 릴렉스 소프트 웨이트바 1kg</t>
+          <t>[1&amp;1] 서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>41,800</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>35,600</t>
+          <t>16,900</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>692</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6664&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17424&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>EKPRB-04</t>
+          <t>EPTSC-05</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>릴렉스 3레벨 스트레칭 롱밴드</t>
+          <t>필라테스 앵클 삭스</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>34,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>34,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>463</t>
+          <t>26</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17424&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6664&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>EPTSC-05</t>
+          <t>EKPRB-04</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>필라테스 앵클 삭스</t>
+          <t>릴렉스 3레벨 스트레칭 롱밴드</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>34,900</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>34,900</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>463</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8837&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>EMTSV-02</t>
+          <t>ENTSC-13</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>[1&amp;1] 서포트 발목 보호대</t>
+          <t>논슬립 퍼포먼스 크루삭스</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>16,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>692</t>
+          <t>659</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -5039,37 +5039,37 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>ENTSC-13</t>
+          <t>ENTSC-19</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 크루삭스</t>
+          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>37%</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>659</t>
+          <t>293</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>ENTSC-19</t>
+          <t>EOTSC-14</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -5123,42 +5123,42 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>EOTSC-14</t>
+          <t>EMTSC-04</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
+          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>293</t>
+          <t>641</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -5195,7 +5195,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>745</t>
+          <t>746</t>
         </is>
       </c>
       <c r="H114" t="inlineStr">
@@ -5207,84 +5207,84 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17440&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>EMTSC-04</t>
+          <t>EPTET-03</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
+          <t>안다르 3단 양우산</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>641</t>
+          <t>34</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.4</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17440&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8836&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>EPTET-03</t>
+          <t>EMTSV-01</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>안다르 3단 양우산</t>
+          <t>[1&amp;1] 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>16,900</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>583</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>593</t>
+          <t>594</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -5417,27 +5417,27 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6665&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13851&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EKPRB-05</t>
+          <t>EOTCP-03</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>릴렉스 4레벨 힙 밴드</t>
+          <t>쿨 라운드 볼캡</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5447,7 +5447,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>519</t>
+          <t>88</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -5459,27 +5459,27 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9988&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6665&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EMTSC-26</t>
+          <t>EKPRB-05</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>램스울 크루 삭스</t>
+          <t>릴렉스 4레벨 힙 밴드</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>292</t>
+          <t>520</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -5501,27 +5501,27 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13851&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9988&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>EOTCP-03</t>
+          <t>EMTSC-26</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>쿨 라운드 볼캡</t>
+          <t>램스울 크루 삭스</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>293</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -5585,37 +5585,37 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16031&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>EOTGL-02</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>[1&amp;1] 3D 쿨링 팔토시</t>
+          <t>히트 런 글러브</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>537</t>
+          <t>209</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -5627,37 +5627,37 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16031&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>EOTGL-02</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>히트 런 글러브</t>
+          <t>[1&amp;1] 3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>537</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>461</t>
+          <t>462</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -5753,79 +5753,79 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8836&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13605&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>EMTSV-01</t>
+          <t>EOTSV-02</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>[1&amp;1] 서포트 팔꿈치 보호대</t>
+          <t>[1&amp;1] 하이 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>16,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>583</t>
+          <t>150</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15867&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13805&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>EOTSC-18</t>
+          <t>EOTSC-04</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>[1&amp;1] 올데이 기모 삭스</t>
+          <t>올데이 수피마 스니커즈 삭스</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>4,500</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>224</t>
+          <t>421</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -5837,37 +5837,37 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13605&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15867&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>EOTSV-02</t>
+          <t>EOTSC-18</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>[1&amp;1] 하이 서포트 팔꿈치 보호대</t>
+          <t>[1&amp;1] 올데이 기모 삭스</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>224</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -5879,84 +5879,84 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13805&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15375&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>EOTSC-04</t>
+          <t>EOTSC-16</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>올데이 수피마 스니커즈 삭스</t>
+          <t>논슬립 스킨 하프 토삭스</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>4,500</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>421</t>
+          <t>96</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15375&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11061&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EOTSC-16</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>논슬립 스킨 하프 토삭스</t>
+          <t>3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>537</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -6047,17 +6047,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11061&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13405&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>EOTSV-01</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>3D 쿨링 팔토시</t>
+          <t>하이 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -6077,7 +6077,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>537</t>
+          <t>672</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -6341,27 +6341,27 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13408&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13831&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>EOTSC-01</t>
+          <t>EOTCP-02</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>프레시 필드 니삭스</t>
+          <t>데님 로고 볼캡</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>290</t>
+          <t>26</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
@@ -6383,37 +6383,37 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13831&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6666&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>EOTCP-02</t>
+          <t>EKPET-01</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>데님 로고 볼캡</t>
+          <t>릴렉스 소프트 웨이트바 1kg</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>19,000</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>590</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -6425,22 +6425,22 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13406&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>EOTSV-02</t>
+          <t>EMTSC-27</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>하이 서포트 팔꿈치 보호대</t>
+          <t>올라운드 오버 니삭스</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -6450,49 +6450,49 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>290</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13408&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>EMTSC-27</t>
+          <t>EOTSC-01</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>올라운드 오버 니삭스</t>
+          <t>프레시 필드 니삭스</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -6502,44 +6502,44 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6666&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13406&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EKPET-01</t>
+          <t>EOTSV-02</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>릴렉스 소프트 웨이트바 1kg</t>
+          <t>하이 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>19,000</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>590</t>
+          <t>150</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
@@ -6677,42 +6677,42 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17387&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>EOTSC-19</t>
+          <t>EPTSC-08</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>[1&amp;1] 레그 워머</t>
+          <t>맨즈 필라테스 크루 삭스</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>229</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
@@ -6724,7 +6724,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>EOTSC-20</t>
+          <t>EOTSC-19</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -6761,42 +6761,42 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17387&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15719&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>EPTSC-08</t>
+          <t>EOTSC-20</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>맨즈 필라테스 크루 삭스</t>
+          <t>[1&amp;1] 레그 워머</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>229</t>
         </is>
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -6845,37 +6845,37 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16035&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17386&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>EOTSC-12</t>
+          <t>EPTSC-07</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>소프트 니트 기모 니삭스</t>
+          <t>맨즈 필라테스 앵클 삭스</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>22%</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
@@ -6887,69 +6887,69 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17386&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12795&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>EPTSC-07</t>
+          <t>ENTCP-05</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>맨즈 필라테스 앵클 삭스</t>
+          <t>소프트 니트 비니</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>22%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>361</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12795&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16035&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>ENTCP-05</t>
+          <t>EOTSC-12</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>소프트 니트 비니</t>
+          <t>소프트 니트 기모 니삭스</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>361</t>
+          <t>101</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
@@ -7001,7 +7001,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>799</t>
+          <t>800</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -7097,111 +7097,111 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11963&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15732&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>ENTSC-19</t>
+          <t>EOTSC-11</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>맨즈 논슬립 하프 토삭스</t>
+          <t>웜 레그 롱 워머</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>113</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16034&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>EPTSC-03</t>
+          <t>EOTGL-03</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>데일리 루즈 삭스</t>
+          <t>소프트 니트 플립 글러브</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>23,900</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>23,900</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>83</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15732&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12792&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>EOTSC-11</t>
+          <t>ENTGL-05</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>웜 레그 롱 워머</t>
+          <t>니트 글러브</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>23,900</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>23,900</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -7211,49 +7211,49 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>366</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16034&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11963&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>EOTGL-03</t>
+          <t>ENTSC-19</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>소프트 니트 플립 글러브</t>
+          <t>맨즈 논슬립 하프 토삭스</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>23,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>23,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>92</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
@@ -7265,27 +7265,27 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12792&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16036&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>ENTGL-05</t>
+          <t>EOTCP-06</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>니트 글러브</t>
+          <t>소프트 니트 버킷햇</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>23,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>23,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -7295,49 +7295,49 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>366</t>
+          <t>52</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16036&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>EOTCP-06</t>
+          <t>EPTSC-03</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>소프트 니트 버킷햇</t>
+          <t>데일리 루즈 삭스</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>21</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -7595,6 +7595,48 @@
       <c r="H171" t="inlineStr">
         <is>
           <t>4.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>https://andar.co.kr/product/detail.html?product_no=11725&amp;cate_no=2100&amp;display_group=1</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>ENTFB-04</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>더블 링글 손목밴드</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>4,900</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>4,900</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>428</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>4.9</t>
         </is>
       </c>
     </row>

</xml_diff>